<commit_message>
result for more tuning added
</commit_message>
<xml_diff>
--- a/hyperparameter_tuning.xlsx
+++ b/hyperparameter_tuning.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\Differentiable-Hydrological-Model-Camels\output\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\Differentiable-Hydrological-Model-Camels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E997845-9CE1-4CC3-85BF-1693AF9DC8E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C4AA511-F621-4805-B519-D57E2F4B48CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-2850" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -139,7 +139,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -159,9 +159,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -458,17 +455,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I35"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="10.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -482,7 +479,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -496,7 +493,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -522,7 +519,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
@@ -548,7 +545,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>256</v>
       </c>
@@ -574,7 +571,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>512</v>
       </c>
@@ -600,7 +597,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>1024</v>
       </c>
@@ -626,7 +623,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3">
         <v>2048</v>
       </c>
@@ -652,7 +649,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
         <f>2048*2</f>
         <v>4096</v>
@@ -680,7 +677,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>0</v>
       </c>
@@ -694,7 +691,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>1</v>
       </c>
@@ -708,7 +705,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>4</v>
       </c>
@@ -734,7 +731,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>3</v>
       </c>
@@ -760,7 +757,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="2">
         <v>128</v>
       </c>
@@ -787,7 +784,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="2">
         <v>256</v>
       </c>
@@ -814,36 +811,36 @@
         <v>56</v>
       </c>
     </row>
-    <row r="18" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="8">
+    <row r="18" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="2">
         <f>128+256</f>
         <v>384</v>
       </c>
-      <c r="B18" s="8">
+      <c r="B18" s="2">
         <v>4.0199999999999996</v>
       </c>
-      <c r="C18" s="8">
+      <c r="C18" s="2">
         <v>172.9</v>
       </c>
-      <c r="D18" s="8">
+      <c r="D18" s="2">
         <v>12</v>
       </c>
       <c r="E18" s="3"/>
-      <c r="F18" s="8">
+      <c r="F18" s="2">
         <f>128+256</f>
         <v>384</v>
       </c>
-      <c r="G18" s="8">
+      <c r="G18" s="2">
         <v>3.31</v>
       </c>
-      <c r="H18" s="8">
+      <c r="H18" s="2">
         <v>379.23</v>
       </c>
-      <c r="I18" s="8">
+      <c r="I18" s="2">
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" s="3">
         <v>512</v>
       </c>
@@ -870,7 +867,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" s="2">
         <v>1024</v>
       </c>
@@ -897,16 +894,22 @@
         <v>30</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="F21" s="2">
         <f>1024*2</f>
         <v>2048</v>
       </c>
-      <c r="G21" s="2"/>
-      <c r="H21" s="2"/>
-      <c r="I21" s="2"/>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G21" s="2">
+        <v>3.26</v>
+      </c>
+      <c r="H21" s="2">
+        <v>542.23</v>
+      </c>
+      <c r="I21" s="2">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>0</v>
       </c>
@@ -914,7 +917,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>1</v>
       </c>
@@ -922,7 +925,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>4</v>
       </c>
@@ -936,7 +939,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>3</v>
       </c>
@@ -950,7 +953,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" s="2">
         <v>2028</v>
       </c>
@@ -964,7 +967,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>0</v>
       </c>
@@ -972,7 +975,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>1</v>
       </c>
@@ -980,7 +983,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>4</v>
       </c>
@@ -994,7 +997,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>3</v>
       </c>
@@ -1008,7 +1011,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35" s="2">
         <v>384</v>
       </c>

</xml_diff>